<commit_message>
Fix: Carrier-Übergabe von +1 TAG auf +2 TAGE korrigiert
User-Anforderung: Logistik-Realität ist 2 Tage Differenz zwischen
Kommissionierung und Carrier-Übergabe, nicht 1 Tag.

Änderung in 6 jtl_text-Templates (kundenseitig, Englisch):
  Lieferung + ohne Terminwunsch + ZAHLUNGSZIEL × {7,14,21 Tage}
                                × {ohne, mit Hebebühne}
  → '[KOMMISSIONIERUNGSTERMIN + 1 TAG]' wird zu
    '[KOMMISSIONIERUNGSTERMIN + 2 TAGE]'

Synchron in allen drei Quellen aktualisiert:
- elvinci_auftragssteuerung.html (Inline JTL_DATA): 6 Stellen
- data/jtl_data.json: 6 Stellen
- data/JTL_Rechnungstexte.xlsx (sheet1 = 'Lieferung OHNE Terminwunsch'): 6 Stellen

XLSX-Repack: ZipArchive-API mit Forward-Slashes (statt Compress-Archive,
das Backslashes erzeugt und XLSX bricht). Inhaltsstruktur identisch zum
Original — nur Texte geändert.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/JTL_Rechnungstexte.xlsx
+++ b/data/JTL_Rechnungstexte.xlsx
@@ -780,7 +780,7 @@
 -	Transport insurance for the net value of the goods is included
 -	ADSp 2017 apply in their current version (https://www.dslv.org/de/adsp)
 Deviations from the above information, lack of availability of a contact person or lack of access at the time of delivery may result in additional cost, which you will be responsible for.
-Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 1 TAG]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
+Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 2 TAGE]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
 You have a payment term of 7 days, which starts from the day the goods are made available for pickup. Please be advised that we reduce your payment term by 7 days for each invoice which is not paid in time.
 TIP: Since October 2025, real-time transfers throughout Europe cost the same as normal SEPA transfers. In many other countries outside Europe, this cost adjustment has also already been implemented or there is at least a transition schedule. If possible, please make your transfer a real-time transfer to ensure that you do not exceed the latest payment date.</t>
         </is>
@@ -850,7 +850,7 @@
 -	Transport insurance for the net value of the goods is included
 -	ADSp 2017 apply in their current version (https://www.dslv.org/de/adsp)
 Deviations from the above information, lack of availability of a contact person or lack of access at the time of delivery may result in additional cost, which you will be responsible for.
-Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 1 TAG]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
+Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 2 TAGE]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
 You have a payment term of 14 days, which starts from the day the goods are made available for pickup. Please be advised that we reduce your payment term by 7 days for each invoice which is not paid in time.
 TIP: Since October 2025, real-time transfers throughout Europe cost the same as normal SEPA transfers. In many other countries outside Europe, this cost adjustment has also already been implemented or there is at least a transition schedule. If possible, please make your transfer a real-time transfer to ensure that you do not exceed the latest payment date.</t>
         </is>
@@ -920,7 +920,7 @@
 -	Transport insurance for the net value of the goods is included
 -	ADSp 2017 apply in their current version (https://www.dslv.org/de/adsp)
 Deviations from the above information, lack of availability of a contact person or lack of access at the time of delivery may result in additional cost, which you will be responsible for.
-Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 1 TAG]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
+Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 2 TAGE]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
 You have a payment term of 21 days, which starts from the day the goods are made available for pickup. Please be advised that we reduce your payment term by 7 days for each invoice which is not paid in time.
 TIP: Since October 2025, real-time transfers throughout Europe cost the same as normal SEPA transfers. In many other countries outside Europe, this cost adjustment has also already been implemented or there is at least a transition schedule. If possible, please make your transfer a real-time transfer to ensure that you do not exceed the latest payment date.</t>
         </is>
@@ -1127,7 +1127,7 @@
 -	Transport insurance for the net value of the goods is included
 -	ADSp 2017 apply in their current version (https://www.dslv.org/de/adsp)
 Deviations from the above information, lack of availability of a contact person or lack of access at the time of delivery may result in additional cost, which you will be responsible for.
-Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 1 TAG]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
+Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 2 TAGE]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
 You have a payment term of 7 days, which starts from the day the goods are made available for pickup. Please be advised that we reduce your payment term by 7 days for each invoice which is not paid in time.
 TIP: Since October 2025, real-time transfers throughout Europe cost the same as normal SEPA transfers. In many other countries outside Europe, this cost adjustment has also already been implemented or there is at least a transition schedule. If possible, please make your transfer a real-time transfer to ensure that you do not exceed the latest payment date.</t>
         </is>
@@ -1197,7 +1197,7 @@
 -	Transport insurance for the net value of the goods is included
 -	ADSp 2017 apply in their current version (https://www.dslv.org/de/adsp)
 Deviations from the above information, lack of availability of a contact person or lack of access at the time of delivery may result in additional cost, which you will be responsible for.
-Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 1 TAG]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
+Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 2 TAGE]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
 You have a payment term of 14 days, which starts from the day the goods are made available for pickup. Please be advised that we reduce your payment term by 7 days for each invoice which is not paid in time.
 TIP: Since October 2025, real-time transfers throughout Europe cost the same as normal SEPA transfers. In many other countries outside Europe, this cost adjustment has also already been implemented or there is at least a transition schedule. If possible, please make your transfer a real-time transfer to ensure that you do not exceed the latest payment date.</t>
         </is>
@@ -1267,7 +1267,7 @@
 -	Transport insurance for the net value of the goods is included
 -	ADSp 2017 apply in their current version (https://www.dslv.org/de/adsp)
 Deviations from the above information, lack of availability of a contact person or lack of access at the time of delivery may result in additional cost, which you will be responsible for.
-Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 1 TAG]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
+Your goods are scheduled for packaging on [KOMMISSIONIERUNGSTERMIN], and will be handed over to the carrier on [KOMMISSIONIERUNGSTERMIN + 2 TAGE]. If you need a fixed delivery date, please contact us by sending an email to info@elvinci.de.
 You have a payment term of 21 days, which starts from the day the goods are made available for pickup. Please be advised that we reduce your payment term by 7 days for each invoice which is not paid in time.
 TIP: Since October 2025, real-time transfers throughout Europe cost the same as normal SEPA transfers. In many other countries outside Europe, this cost adjustment has also already been implemented or there is at least a transition schedule. If possible, please make your transfer a real-time transfer to ensure that you do not exceed the latest payment date.</t>
         </is>

</xml_diff>